<commit_message>
agregando diagrama de flujo y editando inventario en clase
</commit_message>
<xml_diff>
--- a/algoritmos/archivos/datos.xlsx
+++ b/algoritmos/archivos/datos.xlsx
@@ -392,7 +392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,23 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>Jutiapa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Erick</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Jalapa</t>
         </is>
       </c>
     </row>
@@ -474,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,6 +588,29 @@
       </c>
       <c r="E4" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Lenovo</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregando nuevo descuento hecho en clase
</commit_message>
<xml_diff>
--- a/algoritmos/archivos/datos.xlsx
+++ b/algoritmos/archivos/datos.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -611,6 +611,32 @@
       </c>
       <c r="E5" t="n">
         <v>3000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>200</v>
+      </c>
+      <c r="F6" t="n">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>